<commit_message>
Pasar a la peluquería los ejemplos que resolvían casos de las parejas
La ficha de ejemplo, las propuestas de la matriz, el indicador y la
versión A/B usaban la oficina o el comercio, dos de los casos que eligen
las parejas. Cambiados en el guion, en Curso.pptx (diapositivas 65, 66,
73, 87, 97 y 100), en la hoja «Ejemplo» de la matriz y en la pista del
documento del proyecto. Las puntuaciones no cambian: 4,35; 3,30; 4,20.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantillas/matriz_decision.xlsx
+++ b/plantillas/matriz_decision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\Creatividad IA\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B59543-8C59-4BD4-A2E5-4E5D8331E281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEDA2B65-F510-47AD-9ABA-B2A4D899B8E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -188,19 +188,19 @@
     <t>Ejemplo</t>
   </si>
   <si>
-    <t>Formulario digital</t>
-  </si>
-  <si>
-    <t>Propuestas de la explicación del bloque 3. Los datos son supuestos didácticos.</t>
-  </si>
-  <si>
-    <t>Chatbot informativo</t>
-  </si>
-  <si>
     <t>Comprobación a mano: 4×0,35 + 5×0,30 + 5×0,20 + 3×0,15 = 4,35.</t>
   </si>
   <si>
-    <t>Panel de seguimiento</t>
+    <t>Reserva por internet</t>
+  </si>
+  <si>
+    <t>Turno visible en el móvil</t>
+  </si>
+  <si>
+    <t>Abono con cita fija</t>
+  </si>
+  <si>
+    <t>Propuestas del ejemplo de la peluquería (bloque 3). Los datos son supuestos didácticos.</t>
   </si>
 </sst>
 </file>
@@ -864,7 +864,7 @@
     </row>
     <row r="2" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B2" s="5">
         <v>4</v>
@@ -883,7 +883,7 @@
         <v>4.3499999999999996</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -907,12 +907,12 @@
         <v>3.3</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" s="5">
         <v>5</v>

</xml_diff>